<commit_message>
CI + output tables
</commit_message>
<xml_diff>
--- a/output/analysis_output.xlsx
+++ b/output/analysis_output.xlsx
@@ -1,17 +1,17 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="ADF VIF Diagnostics" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="Model Fit" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="Variance Decomposition" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="Wald Joint Tests" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet name="Standardized  Coefficients" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ADF VIF Diagnostics" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Model Fit" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Variance Decomposition" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Wald Joint Tests" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Beta &amp; Confidence Intervals" sheetId="5" state="visible" r:id="rId5"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -1798,373 +1798,928 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I13"/>
+  <dimension ref="A1:W15"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="26" customWidth="1" min="1" max="1"/>
     <col width="16" customWidth="1" min="2" max="2"/>
     <col width="10" customWidth="1" min="3" max="3"/>
-    <col width="13" customWidth="1" min="4" max="4"/>
-    <col width="10" customWidth="1" min="5" max="5"/>
-    <col width="16" customWidth="1" min="6" max="6"/>
-    <col width="13" customWidth="1" min="7" max="7"/>
-    <col width="10" customWidth="1" min="8" max="8"/>
-    <col width="13" customWidth="1" min="9" max="9"/>
+    <col width="11" customWidth="1" min="4" max="4"/>
+    <col width="11" customWidth="1" min="5" max="5"/>
+    <col width="10" customWidth="1" min="6" max="6"/>
+    <col width="11" customWidth="1" min="7" max="7"/>
+    <col width="11" customWidth="1" min="8" max="8"/>
+    <col width="10" customWidth="1" min="9" max="9"/>
+    <col width="11" customWidth="1" min="10" max="10"/>
+    <col width="11" customWidth="1" min="11" max="11"/>
+    <col width="10" customWidth="1" min="12" max="12"/>
+    <col width="11" customWidth="1" min="13" max="13"/>
+    <col width="11" customWidth="1" min="14" max="14"/>
+    <col width="10" customWidth="1" min="15" max="15"/>
+    <col width="11" customWidth="1" min="16" max="16"/>
+    <col width="11" customWidth="1" min="17" max="17"/>
+    <col width="10" customWidth="1" min="18" max="18"/>
+    <col width="11" customWidth="1" min="19" max="19"/>
+    <col width="11" customWidth="1" min="20" max="20"/>
+    <col width="10" customWidth="1" min="21" max="21"/>
+    <col width="11" customWidth="1" min="22" max="22"/>
+    <col width="11" customWidth="1" min="23" max="23"/>
   </cols>
   <sheetData>
     <row r="1" ht="28" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Standardized Factor Transmission Coefficients (β)</t>
-        </is>
-      </c>
-    </row>
-    <row r="2" ht="54" customHeight="1">
+          <t>Beta &amp; 95% HAC Confidence Intervals for Transmission Coefficients</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="30" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Standardized OLS regression coefficients (β) reflecting the marginal impact of macroeconomic predictors on Bursa Malaysia sector returns. Standard errors are adjusted for heteroskedasticity and autocorrelation using Newey-West (HAC) covariance estimation.</t>
+          <t>Point estimates (β), HAC standard errors, and 95% confidence intervals (2.5% to 97.5%) for macroeconomic predictors across KLCI and Bursa Malaysia sector models.</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="3" t="inlineStr">
+      <c r="A4" s="3" t="n"/>
+      <c r="B4" s="3" t="inlineStr">
+        <is>
+          <t>Indices</t>
+        </is>
+      </c>
+      <c r="C4" s="4" t="inlineStr">
+        <is>
+          <t>KLCI</t>
+        </is>
+      </c>
+      <c r="D4" s="4" t="n"/>
+      <c r="E4" s="4" t="n"/>
+      <c r="F4" s="3" t="inlineStr">
+        <is>
+          <t>financials</t>
+        </is>
+      </c>
+      <c r="G4" s="3" t="n"/>
+      <c r="H4" s="3" t="n"/>
+      <c r="I4" s="4" t="inlineStr">
+        <is>
+          <t>energy</t>
+        </is>
+      </c>
+      <c r="J4" s="4" t="n"/>
+      <c r="K4" s="4" t="n"/>
+      <c r="L4" s="3" t="inlineStr">
+        <is>
+          <t>industrial_products</t>
+        </is>
+      </c>
+      <c r="M4" s="3" t="n"/>
+      <c r="N4" s="3" t="n"/>
+      <c r="O4" s="4" t="inlineStr">
+        <is>
+          <t>plantation</t>
+        </is>
+      </c>
+      <c r="P4" s="4" t="n"/>
+      <c r="Q4" s="4" t="n"/>
+      <c r="R4" s="3" t="inlineStr">
+        <is>
+          <t>REITs</t>
+        </is>
+      </c>
+      <c r="S4" s="3" t="n"/>
+      <c r="T4" s="3" t="n"/>
+      <c r="U4" s="4" t="inlineStr">
+        <is>
+          <t>technology</t>
+        </is>
+      </c>
+      <c r="V4" s="4" t="n"/>
+      <c r="W4" s="4" t="n"/>
+    </row>
+    <row r="5">
+      <c r="A5" s="3" t="n"/>
+      <c r="B5" s="3" t="inlineStr">
+        <is>
+          <t>Metrics</t>
+        </is>
+      </c>
+      <c r="C5" s="4" t="inlineStr">
+        <is>
+          <t>beta</t>
+        </is>
+      </c>
+      <c r="D5" s="4" t="inlineStr">
+        <is>
+          <t>CI_lower</t>
+        </is>
+      </c>
+      <c r="E5" s="4" t="inlineStr">
+        <is>
+          <t>CI_upper</t>
+        </is>
+      </c>
+      <c r="F5" s="3" t="inlineStr">
+        <is>
+          <t>beta</t>
+        </is>
+      </c>
+      <c r="G5" s="3" t="inlineStr">
+        <is>
+          <t>CI_lower</t>
+        </is>
+      </c>
+      <c r="H5" s="3" t="inlineStr">
+        <is>
+          <t>CI_upper</t>
+        </is>
+      </c>
+      <c r="I5" s="4" t="inlineStr">
+        <is>
+          <t>beta</t>
+        </is>
+      </c>
+      <c r="J5" s="4" t="inlineStr">
+        <is>
+          <t>CI_lower</t>
+        </is>
+      </c>
+      <c r="K5" s="4" t="inlineStr">
+        <is>
+          <t>CI_upper</t>
+        </is>
+      </c>
+      <c r="L5" s="3" t="inlineStr">
+        <is>
+          <t>beta</t>
+        </is>
+      </c>
+      <c r="M5" s="3" t="inlineStr">
+        <is>
+          <t>CI_lower</t>
+        </is>
+      </c>
+      <c r="N5" s="3" t="inlineStr">
+        <is>
+          <t>CI_upper</t>
+        </is>
+      </c>
+      <c r="O5" s="4" t="inlineStr">
+        <is>
+          <t>beta</t>
+        </is>
+      </c>
+      <c r="P5" s="4" t="inlineStr">
+        <is>
+          <t>CI_lower</t>
+        </is>
+      </c>
+      <c r="Q5" s="4" t="inlineStr">
+        <is>
+          <t>CI_upper</t>
+        </is>
+      </c>
+      <c r="R5" s="3" t="inlineStr">
+        <is>
+          <t>beta</t>
+        </is>
+      </c>
+      <c r="S5" s="3" t="inlineStr">
+        <is>
+          <t>CI_lower</t>
+        </is>
+      </c>
+      <c r="T5" s="3" t="inlineStr">
+        <is>
+          <t>CI_upper</t>
+        </is>
+      </c>
+      <c r="U5" s="4" t="inlineStr">
+        <is>
+          <t>beta</t>
+        </is>
+      </c>
+      <c r="V5" s="4" t="inlineStr">
+        <is>
+          <t>CI_lower</t>
+        </is>
+      </c>
+      <c r="W5" s="4" t="inlineStr">
+        <is>
+          <t>CI_upper</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="3" t="inlineStr">
         <is>
           <t>Channels</t>
         </is>
       </c>
-      <c r="B4" s="3" t="inlineStr">
+      <c r="B6" s="3" t="inlineStr">
         <is>
           <t>Variables</t>
         </is>
       </c>
-      <c r="C4" s="3" t="inlineStr">
-        <is>
-          <t>KLCI</t>
-        </is>
-      </c>
-      <c r="D4" s="3" t="inlineStr">
-        <is>
-          <t>financials</t>
-        </is>
-      </c>
-      <c r="E4" s="3" t="inlineStr">
-        <is>
-          <t>energy</t>
-        </is>
-      </c>
-      <c r="F4" s="3" t="inlineStr">
-        <is>
-          <t>industrial_products</t>
-        </is>
-      </c>
-      <c r="G4" s="3" t="inlineStr">
-        <is>
-          <t>plantation</t>
-        </is>
-      </c>
-      <c r="H4" s="3" t="inlineStr">
-        <is>
-          <t>REITs</t>
-        </is>
-      </c>
-      <c r="I4" s="3" t="inlineStr">
-        <is>
-          <t>technology</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" s="4" t="inlineStr">
+      <c r="C6" s="4" t="n"/>
+      <c r="D6" s="4" t="n"/>
+      <c r="E6" s="4" t="n"/>
+      <c r="F6" s="3" t="n"/>
+      <c r="G6" s="3" t="n"/>
+      <c r="H6" s="3" t="n"/>
+      <c r="I6" s="4" t="n"/>
+      <c r="J6" s="4" t="n"/>
+      <c r="K6" s="4" t="n"/>
+      <c r="L6" s="3" t="n"/>
+      <c r="M6" s="3" t="n"/>
+      <c r="N6" s="3" t="n"/>
+      <c r="O6" s="4" t="n"/>
+      <c r="P6" s="4" t="n"/>
+      <c r="Q6" s="4" t="n"/>
+      <c r="R6" s="3" t="n"/>
+      <c r="S6" s="3" t="n"/>
+      <c r="T6" s="3" t="n"/>
+      <c r="U6" s="4" t="n"/>
+      <c r="V6" s="4" t="n"/>
+      <c r="W6" s="4" t="n"/>
+    </row>
+    <row r="7">
+      <c r="A7" s="4" t="inlineStr">
         <is>
           <t>Domestic Baseline</t>
         </is>
       </c>
-      <c r="B5" s="4" t="inlineStr">
+      <c r="B7" s="4" t="inlineStr">
         <is>
           <t>cpi_inflation</t>
         </is>
       </c>
-      <c r="C5" s="5" t="n">
+      <c r="C7" s="5" t="n">
         <v>-0.5482423421184817</v>
       </c>
-      <c r="D5" s="5" t="n">
+      <c r="D7" s="5" t="n">
+        <v>-1.541725857874326</v>
+      </c>
+      <c r="E7" s="5" t="n">
+        <v>0.4452411736373632</v>
+      </c>
+      <c r="F7" s="5" t="n">
         <v>0.2618790981863163</v>
       </c>
-      <c r="E5" s="5" t="n">
+      <c r="G7" s="5" t="n">
+        <v>-1.241497356439079</v>
+      </c>
+      <c r="H7" s="5" t="n">
+        <v>1.765255552811711</v>
+      </c>
+      <c r="I7" s="5" t="n">
         <v>-1.968836043767184</v>
       </c>
-      <c r="F5" s="5" t="n">
+      <c r="J7" s="5" t="n">
+        <v>-3.671718131445655</v>
+      </c>
+      <c r="K7" s="5" t="n">
+        <v>-0.2659539560887143</v>
+      </c>
+      <c r="L7" s="5" t="n">
         <v>-1.08749923244575</v>
       </c>
-      <c r="G5" s="5" t="n">
+      <c r="M7" s="5" t="n">
+        <v>-6.053568293348436</v>
+      </c>
+      <c r="N7" s="5" t="n">
+        <v>3.878569828456935</v>
+      </c>
+      <c r="O7" s="5" t="n">
         <v>-0.660968084728121</v>
       </c>
-      <c r="H5" s="5" t="n">
+      <c r="P7" s="5" t="n">
+        <v>-2.597605518485457</v>
+      </c>
+      <c r="Q7" s="5" t="n">
+        <v>1.275669349029215</v>
+      </c>
+      <c r="R7" s="5" t="n">
         <v>0.6992802674585527</v>
       </c>
-      <c r="I5" s="5" t="n">
+      <c r="S7" s="5" t="n">
+        <v>-0.3296216144376013</v>
+      </c>
+      <c r="T7" s="5" t="n">
+        <v>1.728182149354707</v>
+      </c>
+      <c r="U7" s="5" t="n">
         <v>1.632130213666181</v>
       </c>
-    </row>
-    <row r="6">
-      <c r="A6" s="4" t="n"/>
-      <c r="B6" s="4" t="inlineStr">
+      <c r="V7" s="5" t="n">
+        <v>-1.415682567705457</v>
+      </c>
+      <c r="W7" s="5" t="n">
+        <v>4.67994299503782</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="4" t="n"/>
+      <c r="B8" s="4" t="inlineStr">
         <is>
           <t>IPI</t>
         </is>
       </c>
-      <c r="C6" s="5" t="n">
+      <c r="C8" s="5" t="n">
         <v>0.0002729301239610855</v>
       </c>
-      <c r="D6" s="5" t="n">
+      <c r="D8" s="5" t="n">
+        <v>-0.0002336994774122813</v>
+      </c>
+      <c r="E8" s="5" t="n">
+        <v>0.0007795597253344524</v>
+      </c>
+      <c r="F8" s="5" t="n">
         <v>0.0002424318847966879</v>
       </c>
-      <c r="E6" s="5" t="n">
+      <c r="G8" s="5" t="n">
+        <v>-0.00028465629453139</v>
+      </c>
+      <c r="H8" s="5" t="n">
+        <v>0.0007695200641247657</v>
+      </c>
+      <c r="I8" s="5" t="n">
         <v>-0.0002745589580463794</v>
       </c>
-      <c r="F6" s="5" t="n">
+      <c r="J8" s="5" t="n">
+        <v>-0.001166546185215082</v>
+      </c>
+      <c r="K8" s="5" t="n">
+        <v>0.0006174282691223228</v>
+      </c>
+      <c r="L8" s="5" t="n">
         <v>-1.293322461919992e-06</v>
       </c>
-      <c r="G6" s="5" t="n">
+      <c r="M8" s="5" t="n">
+        <v>-0.002713825801965323</v>
+      </c>
+      <c r="N8" s="5" t="n">
+        <v>0.002711239157041483</v>
+      </c>
+      <c r="O8" s="5" t="n">
         <v>0.0008794828932350875</v>
       </c>
-      <c r="H6" s="5" t="n">
+      <c r="P8" s="5" t="n">
+        <v>-0.0003107812168985434</v>
+      </c>
+      <c r="Q8" s="5" t="n">
+        <v>0.002069747003368718</v>
+      </c>
+      <c r="R8" s="5" t="n">
         <v>-0.0004406723349784292</v>
       </c>
-      <c r="I6" s="5" t="n">
+      <c r="S8" s="5" t="n">
+        <v>-0.001223392685203437</v>
+      </c>
+      <c r="T8" s="5" t="n">
+        <v>0.0003420480152465782</v>
+      </c>
+      <c r="U8" s="5" t="n">
         <v>-0.0003112903627832451</v>
       </c>
-    </row>
-    <row r="7">
-      <c r="A7" s="3" t="inlineStr">
-        <is>
-          <t>Rate Differential</t>
-        </is>
-      </c>
-      <c r="B7" s="3" t="inlineStr">
-        <is>
-          <t>FFR_OPR_diff</t>
-        </is>
-      </c>
-      <c r="C7" s="6" t="n">
-        <v>-0.0120438960910971</v>
-      </c>
-      <c r="D7" s="6" t="n">
-        <v>-0.003217276961140139</v>
-      </c>
-      <c r="E7" s="6" t="n">
-        <v>-0.01354486073883431</v>
-      </c>
-      <c r="F7" s="6" t="n">
-        <v>-0.05676428376993873</v>
-      </c>
-      <c r="G7" s="6" t="n">
-        <v>-0.04954613454682324</v>
-      </c>
-      <c r="H7" s="6" t="n">
-        <v>0.02272648726281115</v>
-      </c>
-      <c r="I7" s="6" t="n">
-        <v>0.001779703779848962</v>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" s="4" t="inlineStr">
-        <is>
-          <t>Global Risk Appetite</t>
-        </is>
-      </c>
-      <c r="B8" s="4" t="inlineStr">
-        <is>
-          <t>VIX</t>
-        </is>
-      </c>
-      <c r="C8" s="5" t="n">
-        <v>-0.0004851976036206086</v>
-      </c>
-      <c r="D8" s="5" t="n">
-        <v>-0.000826195660979923</v>
-      </c>
-      <c r="E8" s="5" t="n">
-        <v>-0.001001619124555685</v>
-      </c>
-      <c r="F8" s="5" t="n">
-        <v>0.0006516030606860851</v>
-      </c>
-      <c r="G8" s="5" t="n">
-        <v>-4.948763045824571e-05</v>
-      </c>
-      <c r="H8" s="5" t="n">
-        <v>-0.0002660068688006391</v>
-      </c>
-      <c r="I8" s="5" t="n">
-        <v>-0.002713913057161963</v>
+      <c r="V8" s="5" t="n">
+        <v>-0.00272779694097448</v>
+      </c>
+      <c r="W8" s="5" t="n">
+        <v>0.00210521621540799</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="3" t="inlineStr">
         <is>
+          <t>Rate Differential</t>
+        </is>
+      </c>
+      <c r="B9" s="3" t="inlineStr">
+        <is>
+          <t>FFR_OPR_diff</t>
+        </is>
+      </c>
+      <c r="C9" s="5" t="n">
+        <v>-0.0120438960910971</v>
+      </c>
+      <c r="D9" s="5" t="n">
+        <v>-0.03914678716199117</v>
+      </c>
+      <c r="E9" s="5" t="n">
+        <v>0.01505899497979697</v>
+      </c>
+      <c r="F9" s="6" t="n">
+        <v>-0.003217276961140139</v>
+      </c>
+      <c r="G9" s="6" t="n">
+        <v>-0.03032001839346419</v>
+      </c>
+      <c r="H9" s="6" t="n">
+        <v>0.02388546447118392</v>
+      </c>
+      <c r="I9" s="5" t="n">
+        <v>-0.01354486073883431</v>
+      </c>
+      <c r="J9" s="5" t="n">
+        <v>-0.05586486084421864</v>
+      </c>
+      <c r="K9" s="5" t="n">
+        <v>0.02877513936655002</v>
+      </c>
+      <c r="L9" s="6" t="n">
+        <v>-0.05676428376993873</v>
+      </c>
+      <c r="M9" s="6" t="n">
+        <v>-0.146027198396996</v>
+      </c>
+      <c r="N9" s="6" t="n">
+        <v>0.03249863085711849</v>
+      </c>
+      <c r="O9" s="5" t="n">
+        <v>-0.04954613454682324</v>
+      </c>
+      <c r="P9" s="5" t="n">
+        <v>-0.1069826481655368</v>
+      </c>
+      <c r="Q9" s="5" t="n">
+        <v>0.007890379071890309</v>
+      </c>
+      <c r="R9" s="6" t="n">
+        <v>0.02272648726281115</v>
+      </c>
+      <c r="S9" s="6" t="n">
+        <v>-0.006496658296303331</v>
+      </c>
+      <c r="T9" s="6" t="n">
+        <v>0.05194963282192563</v>
+      </c>
+      <c r="U9" s="5" t="n">
+        <v>0.001779703779848962</v>
+      </c>
+      <c r="V9" s="5" t="n">
+        <v>-0.04672758840926379</v>
+      </c>
+      <c r="W9" s="5" t="n">
+        <v>0.05028699596896172</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="4" t="inlineStr">
+        <is>
+          <t>Global Risk Appetite</t>
+        </is>
+      </c>
+      <c r="B10" s="4" t="inlineStr">
+        <is>
+          <t>VIX</t>
+        </is>
+      </c>
+      <c r="C10" s="5" t="n">
+        <v>-0.0004851976036206086</v>
+      </c>
+      <c r="D10" s="5" t="n">
+        <v>-0.001427489147824312</v>
+      </c>
+      <c r="E10" s="5" t="n">
+        <v>0.0004570939405830946</v>
+      </c>
+      <c r="F10" s="5" t="n">
+        <v>-0.000826195660979923</v>
+      </c>
+      <c r="G10" s="5" t="n">
+        <v>-0.002517082529766342</v>
+      </c>
+      <c r="H10" s="5" t="n">
+        <v>0.0008646912078064965</v>
+      </c>
+      <c r="I10" s="5" t="n">
+        <v>-0.001001619124555685</v>
+      </c>
+      <c r="J10" s="5" t="n">
+        <v>-0.002973321477981247</v>
+      </c>
+      <c r="K10" s="5" t="n">
+        <v>0.0009700832288698775</v>
+      </c>
+      <c r="L10" s="5" t="n">
+        <v>0.0006516030606860851</v>
+      </c>
+      <c r="M10" s="5" t="n">
+        <v>-0.002247059131435814</v>
+      </c>
+      <c r="N10" s="5" t="n">
+        <v>0.003550265252807984</v>
+      </c>
+      <c r="O10" s="5" t="n">
+        <v>-4.948763045824571e-05</v>
+      </c>
+      <c r="P10" s="5" t="n">
+        <v>-0.002475607803393917</v>
+      </c>
+      <c r="Q10" s="5" t="n">
+        <v>0.002376632542477425</v>
+      </c>
+      <c r="R10" s="5" t="n">
+        <v>-0.0002660068688006391</v>
+      </c>
+      <c r="S10" s="5" t="n">
+        <v>-0.001611860824041869</v>
+      </c>
+      <c r="T10" s="5" t="n">
+        <v>0.001079847086440591</v>
+      </c>
+      <c r="U10" s="5" t="n">
+        <v>-0.002713913057161963</v>
+      </c>
+      <c r="V10" s="5" t="n">
+        <v>-0.006561771854417833</v>
+      </c>
+      <c r="W10" s="5" t="n">
+        <v>0.001133945740093906</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="3" t="inlineStr">
+        <is>
           <t>Global Credit Condition</t>
         </is>
       </c>
-      <c r="B9" s="3" t="inlineStr">
+      <c r="B11" s="3" t="inlineStr">
         <is>
           <t>UST_10Y</t>
         </is>
       </c>
-      <c r="C9" s="6" t="n">
+      <c r="C11" s="5" t="n">
         <v>0.002347323450798132</v>
       </c>
-      <c r="D9" s="6" t="n">
+      <c r="D11" s="5" t="n">
+        <v>-0.02224254442167136</v>
+      </c>
+      <c r="E11" s="5" t="n">
+        <v>0.02693719132326763</v>
+      </c>
+      <c r="F11" s="6" t="n">
         <v>0.01896011281041776</v>
       </c>
-      <c r="E9" s="6" t="n">
+      <c r="G11" s="6" t="n">
+        <v>-0.007808068322245926</v>
+      </c>
+      <c r="H11" s="6" t="n">
+        <v>0.04572829394308144</v>
+      </c>
+      <c r="I11" s="5" t="n">
         <v>0.01110720076736025</v>
       </c>
-      <c r="F9" s="6" t="n">
+      <c r="J11" s="5" t="n">
+        <v>-0.01827997127370456</v>
+      </c>
+      <c r="K11" s="5" t="n">
+        <v>0.04049437280842505</v>
+      </c>
+      <c r="L11" s="6" t="n">
         <v>-0.05688451707978919</v>
       </c>
-      <c r="G9" s="6" t="n">
+      <c r="M11" s="6" t="n">
+        <v>-0.1198278250631943</v>
+      </c>
+      <c r="N11" s="6" t="n">
+        <v>0.006058790903615906</v>
+      </c>
+      <c r="O11" s="5" t="n">
         <v>0.001783838005130882</v>
       </c>
-      <c r="H9" s="6" t="n">
+      <c r="P11" s="5" t="n">
+        <v>-0.03840240777512716</v>
+      </c>
+      <c r="Q11" s="5" t="n">
+        <v>0.04197008378538893</v>
+      </c>
+      <c r="R11" s="6" t="n">
         <v>-0.03251854003148871</v>
       </c>
-      <c r="I9" s="6" t="n">
+      <c r="S11" s="6" t="n">
+        <v>-0.06073261868674925</v>
+      </c>
+      <c r="T11" s="6" t="n">
+        <v>-0.004304461376228162</v>
+      </c>
+      <c r="U11" s="5" t="n">
         <v>-0.01889481480612774</v>
       </c>
-    </row>
-    <row r="10">
-      <c r="A10" s="3" t="n"/>
-      <c r="B10" s="3" t="inlineStr">
+      <c r="V11" s="5" t="n">
+        <v>-0.07735891032834516</v>
+      </c>
+      <c r="W11" s="5" t="n">
+        <v>0.03956928071608967</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="3" t="n"/>
+      <c r="B12" s="3" t="inlineStr">
         <is>
           <t>HY_OAS</t>
         </is>
       </c>
-      <c r="C10" s="6" t="n">
+      <c r="C12" s="5" t="n">
         <v>-0.0184579755870158</v>
       </c>
-      <c r="D10" s="6" t="n">
+      <c r="D12" s="5" t="n">
+        <v>-0.032062284663861</v>
+      </c>
+      <c r="E12" s="5" t="n">
+        <v>-0.0048536665101706</v>
+      </c>
+      <c r="F12" s="6" t="n">
         <v>-0.01648583523094233</v>
       </c>
-      <c r="E10" s="6" t="n">
+      <c r="G12" s="6" t="n">
+        <v>-0.0314190116494683</v>
+      </c>
+      <c r="H12" s="6" t="n">
+        <v>-0.001552658812416365</v>
+      </c>
+      <c r="I12" s="5" t="n">
         <v>0.01691014377155839</v>
       </c>
-      <c r="F10" s="6" t="n">
+      <c r="J12" s="5" t="n">
+        <v>-0.0108958720644927</v>
+      </c>
+      <c r="K12" s="5" t="n">
+        <v>0.04471615960760948</v>
+      </c>
+      <c r="L12" s="6" t="n">
         <v>-0.04879046560426468</v>
       </c>
-      <c r="G10" s="6" t="n">
+      <c r="M12" s="6" t="n">
+        <v>-0.09136952139527177</v>
+      </c>
+      <c r="N12" s="6" t="n">
+        <v>-0.006211409813257594</v>
+      </c>
+      <c r="O12" s="5" t="n">
         <v>-0.002082114571569562</v>
       </c>
-      <c r="H10" s="6" t="n">
+      <c r="P12" s="5" t="n">
+        <v>-0.03856735295211186</v>
+      </c>
+      <c r="Q12" s="5" t="n">
+        <v>0.03440312380897273</v>
+      </c>
+      <c r="R12" s="6" t="n">
         <v>-0.01246091850018913</v>
       </c>
-      <c r="I10" s="6" t="n">
+      <c r="S12" s="6" t="n">
+        <v>-0.02924813469244573</v>
+      </c>
+      <c r="T12" s="6" t="n">
+        <v>0.004326297692067462</v>
+      </c>
+      <c r="U12" s="5" t="n">
         <v>-0.06684304493937422</v>
       </c>
-    </row>
-    <row r="11">
-      <c r="A11" s="4" t="inlineStr">
+      <c r="V12" s="5" t="n">
+        <v>-0.1035095475778177</v>
+      </c>
+      <c r="W12" s="5" t="n">
+        <v>-0.0301765423009307</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="4" t="inlineStr">
         <is>
           <t>FX Pass-Through</t>
         </is>
       </c>
-      <c r="B11" s="4" t="inlineStr">
+      <c r="B13" s="4" t="inlineStr">
         <is>
           <t>USDMYR</t>
         </is>
       </c>
-      <c r="C11" s="5" t="n">
+      <c r="C13" s="5" t="n">
         <v>-0.3479691930007035</v>
       </c>
-      <c r="D11" s="5" t="n">
+      <c r="D13" s="5" t="n">
+        <v>-0.5593766876458407</v>
+      </c>
+      <c r="E13" s="5" t="n">
+        <v>-0.1365616983555663</v>
+      </c>
+      <c r="F13" s="5" t="n">
         <v>-0.554850971333216</v>
       </c>
-      <c r="E11" s="5" t="n">
+      <c r="G13" s="5" t="n">
+        <v>-0.8809675042797518</v>
+      </c>
+      <c r="H13" s="5" t="n">
+        <v>-0.2287344383866802</v>
+      </c>
+      <c r="I13" s="5" t="n">
         <v>-0.04378003435391339</v>
       </c>
-      <c r="F11" s="5" t="n">
+      <c r="J13" s="5" t="n">
+        <v>-0.4557753430651801</v>
+      </c>
+      <c r="K13" s="5" t="n">
+        <v>0.3682152743573534</v>
+      </c>
+      <c r="L13" s="5" t="n">
         <v>-0.06869547448332119</v>
       </c>
-      <c r="G11" s="5" t="n">
+      <c r="M13" s="5" t="n">
+        <v>-0.7660613520725512</v>
+      </c>
+      <c r="N13" s="5" t="n">
+        <v>0.6286704031059089</v>
+      </c>
+      <c r="O13" s="5" t="n">
         <v>-0.06961261982621557</v>
       </c>
-      <c r="H11" s="5" t="n">
+      <c r="P13" s="5" t="n">
+        <v>-0.5769174265387652</v>
+      </c>
+      <c r="Q13" s="5" t="n">
+        <v>0.437692186886334</v>
+      </c>
+      <c r="R13" s="5" t="n">
         <v>0.03657371716226639</v>
       </c>
-      <c r="I11" s="5" t="n">
+      <c r="S13" s="5" t="n">
+        <v>-0.3564487731097409</v>
+      </c>
+      <c r="T13" s="5" t="n">
+        <v>0.4295962074342737</v>
+      </c>
+      <c r="U13" s="5" t="n">
         <v>0.4663416192881011</v>
       </c>
-    </row>
-    <row r="12">
-      <c r="A12" s="3" t="inlineStr">
+      <c r="V13" s="5" t="n">
+        <v>-0.2860530578119991</v>
+      </c>
+      <c r="W13" s="5" t="n">
+        <v>1.218736296388201</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="3" t="inlineStr">
         <is>
           <t>Commodity</t>
         </is>
       </c>
-      <c r="B12" s="3" t="inlineStr">
+      <c r="B14" s="3" t="inlineStr">
         <is>
           <t>CPO</t>
         </is>
       </c>
-      <c r="C12" s="6" t="n">
+      <c r="C14" s="5" t="n">
         <v>-0.04476067111596965</v>
       </c>
-      <c r="D12" s="6" t="n">
+      <c r="D14" s="5" t="n">
+        <v>-0.09044242857389331</v>
+      </c>
+      <c r="E14" s="5" t="n">
+        <v>0.0009210863419540222</v>
+      </c>
+      <c r="F14" s="6" t="n">
         <v>-0.03101491007731285</v>
       </c>
-      <c r="E12" s="6" t="n">
+      <c r="G14" s="6" t="n">
+        <v>-0.1047056127809043</v>
+      </c>
+      <c r="H14" s="6" t="n">
+        <v>0.04267579262627855</v>
+      </c>
+      <c r="I14" s="5" t="n">
         <v>-0.03388319657228572</v>
       </c>
-      <c r="F12" s="6" t="n">
+      <c r="J14" s="5" t="n">
+        <v>-0.1395923685113756</v>
+      </c>
+      <c r="K14" s="5" t="n">
+        <v>0.07182597536680418</v>
+      </c>
+      <c r="L14" s="6" t="n">
         <v>0.0472199908514435</v>
       </c>
-      <c r="G12" s="6" t="n">
+      <c r="M14" s="6" t="n">
+        <v>-0.1055560673899905</v>
+      </c>
+      <c r="N14" s="6" t="n">
+        <v>0.1999960490928775</v>
+      </c>
+      <c r="O14" s="5" t="n">
         <v>-0.03480524597027135</v>
       </c>
-      <c r="H12" s="6" t="n">
+      <c r="P14" s="5" t="n">
+        <v>-0.1666050098385253</v>
+      </c>
+      <c r="Q14" s="5" t="n">
+        <v>0.09699451789798258</v>
+      </c>
+      <c r="R14" s="6" t="n">
         <v>0.0281414002973919</v>
       </c>
-      <c r="I12" s="6" t="n">
+      <c r="S14" s="6" t="n">
+        <v>-0.02594265594952315</v>
+      </c>
+      <c r="T14" s="6" t="n">
+        <v>0.08222545654430695</v>
+      </c>
+      <c r="U14" s="5" t="n">
         <v>0.08674972761160121</v>
       </c>
-    </row>
-    <row r="13">
-      <c r="A13" s="3" t="n"/>
-      <c r="B13" s="3" t="inlineStr">
+      <c r="V14" s="5" t="n">
+        <v>-0.06970115338726085</v>
+      </c>
+      <c r="W14" s="5" t="n">
+        <v>0.2432006086104633</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="3" t="n"/>
+      <c r="B15" s="3" t="inlineStr">
         <is>
           <t>Oil</t>
         </is>
       </c>
-      <c r="C13" s="6" t="n">
+      <c r="C15" s="5" t="n">
         <v>0.01801504517179942</v>
       </c>
-      <c r="D13" s="6" t="n">
+      <c r="D15" s="5" t="n">
+        <v>-0.01945058345604088</v>
+      </c>
+      <c r="E15" s="5" t="n">
+        <v>0.05548067379963971</v>
+      </c>
+      <c r="F15" s="6" t="n">
         <v>0.02394157441402341</v>
       </c>
-      <c r="E13" s="6" t="n">
+      <c r="G15" s="6" t="n">
+        <v>-0.03469264895659442</v>
+      </c>
+      <c r="H15" s="6" t="n">
+        <v>0.08257579778464123</v>
+      </c>
+      <c r="I15" s="5" t="n">
         <v>0.1940446307095657</v>
       </c>
-      <c r="F13" s="6" t="n">
+      <c r="J15" s="5" t="n">
+        <v>0.02720669959656918</v>
+      </c>
+      <c r="K15" s="5" t="n">
+        <v>0.3608825618225622</v>
+      </c>
+      <c r="L15" s="6" t="n">
         <v>0.06746046882238525</v>
       </c>
-      <c r="G13" s="6" t="n">
+      <c r="M15" s="6" t="n">
+        <v>-0.08277076473970842</v>
+      </c>
+      <c r="N15" s="6" t="n">
+        <v>0.2176917023844789</v>
+      </c>
+      <c r="O15" s="5" t="n">
         <v>0.132076941747987</v>
       </c>
-      <c r="H13" s="6" t="n">
+      <c r="P15" s="5" t="n">
+        <v>0.04811570527043092</v>
+      </c>
+      <c r="Q15" s="5" t="n">
+        <v>0.2160381782255432</v>
+      </c>
+      <c r="R15" s="6" t="n">
         <v>0.02793195311850622</v>
       </c>
-      <c r="I13" s="6" t="n">
+      <c r="S15" s="6" t="n">
+        <v>-0.02097406715310803</v>
+      </c>
+      <c r="T15" s="6" t="n">
+        <v>0.07683797339012048</v>
+      </c>
+      <c r="U15" s="5" t="n">
         <v>-0.1083130738338397</v>
       </c>
+      <c r="V15" s="5" t="n">
+        <v>-0.2215082881820247</v>
+      </c>
+      <c r="W15" s="5" t="n">
+        <v>0.004882140514345226</v>
+      </c>
     </row>
   </sheetData>
-  <mergeCells count="5">
-    <mergeCell ref="A5:A6"/>
-    <mergeCell ref="A2:I2"/>
-    <mergeCell ref="A9:A10"/>
-    <mergeCell ref="A12:A13"/>
-    <mergeCell ref="A1:I1"/>
+  <mergeCells count="12">
+    <mergeCell ref="A1:W1"/>
+    <mergeCell ref="A14:A15"/>
+    <mergeCell ref="O4:Q4"/>
+    <mergeCell ref="R4:T4"/>
+    <mergeCell ref="C4:E4"/>
+    <mergeCell ref="U4:W4"/>
+    <mergeCell ref="F4:H4"/>
+    <mergeCell ref="A7:A8"/>
+    <mergeCell ref="I4:K4"/>
+    <mergeCell ref="L4:N4"/>
+    <mergeCell ref="A2:W2"/>
+    <mergeCell ref="A11:A12"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
CI relative width ratio
</commit_message>
<xml_diff>
--- a/output/analysis_output.xlsx
+++ b/output/analysis_output.xlsx
@@ -1798,7 +1798,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:W15"/>
+  <dimension ref="A1:AD15"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="26" customWidth="1" min="1" max="1"/>
@@ -1806,24 +1806,31 @@
     <col width="10" customWidth="1" min="3" max="3"/>
     <col width="11" customWidth="1" min="4" max="4"/>
     <col width="11" customWidth="1" min="5" max="5"/>
-    <col width="10" customWidth="1" min="6" max="6"/>
-    <col width="11" customWidth="1" min="7" max="7"/>
+    <col width="16" customWidth="1" min="6" max="6"/>
+    <col width="10" customWidth="1" min="7" max="7"/>
     <col width="11" customWidth="1" min="8" max="8"/>
-    <col width="10" customWidth="1" min="9" max="9"/>
-    <col width="11" customWidth="1" min="10" max="10"/>
-    <col width="11" customWidth="1" min="11" max="11"/>
-    <col width="10" customWidth="1" min="12" max="12"/>
+    <col width="11" customWidth="1" min="9" max="9"/>
+    <col width="16" customWidth="1" min="10" max="10"/>
+    <col width="10" customWidth="1" min="11" max="11"/>
+    <col width="11" customWidth="1" min="12" max="12"/>
     <col width="11" customWidth="1" min="13" max="13"/>
-    <col width="11" customWidth="1" min="14" max="14"/>
+    <col width="16" customWidth="1" min="14" max="14"/>
     <col width="10" customWidth="1" min="15" max="15"/>
     <col width="11" customWidth="1" min="16" max="16"/>
     <col width="11" customWidth="1" min="17" max="17"/>
-    <col width="10" customWidth="1" min="18" max="18"/>
-    <col width="11" customWidth="1" min="19" max="19"/>
+    <col width="16" customWidth="1" min="18" max="18"/>
+    <col width="10" customWidth="1" min="19" max="19"/>
     <col width="11" customWidth="1" min="20" max="20"/>
-    <col width="10" customWidth="1" min="21" max="21"/>
-    <col width="11" customWidth="1" min="22" max="22"/>
-    <col width="11" customWidth="1" min="23" max="23"/>
+    <col width="11" customWidth="1" min="21" max="21"/>
+    <col width="16" customWidth="1" min="22" max="22"/>
+    <col width="10" customWidth="1" min="23" max="23"/>
+    <col width="11" customWidth="1" min="24" max="24"/>
+    <col width="11" customWidth="1" min="25" max="25"/>
+    <col width="16" customWidth="1" min="26" max="26"/>
+    <col width="10" customWidth="1" min="27" max="27"/>
+    <col width="11" customWidth="1" min="28" max="28"/>
+    <col width="11" customWidth="1" min="29" max="29"/>
+    <col width="16" customWidth="1" min="30" max="30"/>
   </cols>
   <sheetData>
     <row r="1" ht="28" customHeight="1">
@@ -1854,56 +1861,59 @@
       </c>
       <c r="D4" s="4" t="n"/>
       <c r="E4" s="4" t="n"/>
-      <c r="F4" s="3" t="inlineStr">
+      <c r="F4" s="4" t="n"/>
+      <c r="G4" s="3" t="inlineStr">
         <is>
           <t>financials</t>
         </is>
       </c>
-      <c r="G4" s="3" t="n"/>
       <c r="H4" s="3" t="n"/>
-      <c r="I4" s="4" t="inlineStr">
+      <c r="I4" s="3" t="n"/>
+      <c r="J4" s="3" t="n"/>
+      <c r="K4" s="4" t="inlineStr">
         <is>
           <t>energy</t>
         </is>
       </c>
-      <c r="J4" s="4" t="n"/>
-      <c r="K4" s="4" t="n"/>
-      <c r="L4" s="3" t="inlineStr">
+      <c r="L4" s="4" t="n"/>
+      <c r="M4" s="4" t="n"/>
+      <c r="N4" s="4" t="n"/>
+      <c r="O4" s="3" t="inlineStr">
         <is>
           <t>industrial_products</t>
         </is>
       </c>
-      <c r="M4" s="3" t="n"/>
-      <c r="N4" s="3" t="n"/>
-      <c r="O4" s="4" t="inlineStr">
+      <c r="P4" s="3" t="n"/>
+      <c r="Q4" s="3" t="n"/>
+      <c r="R4" s="3" t="n"/>
+      <c r="S4" s="4" t="inlineStr">
         <is>
           <t>plantation</t>
         </is>
       </c>
-      <c r="P4" s="4" t="n"/>
-      <c r="Q4" s="4" t="n"/>
-      <c r="R4" s="3" t="inlineStr">
+      <c r="T4" s="4" t="n"/>
+      <c r="U4" s="4" t="n"/>
+      <c r="V4" s="4" t="n"/>
+      <c r="W4" s="3" t="inlineStr">
         <is>
           <t>REITs</t>
         </is>
       </c>
-      <c r="S4" s="3" t="n"/>
-      <c r="T4" s="3" t="n"/>
-      <c r="U4" s="4" t="inlineStr">
+      <c r="X4" s="3" t="n"/>
+      <c r="Y4" s="3" t="n"/>
+      <c r="Z4" s="3" t="n"/>
+      <c r="AA4" s="4" t="inlineStr">
         <is>
           <t>technology</t>
         </is>
       </c>
-      <c r="V4" s="4" t="n"/>
-      <c r="W4" s="4" t="n"/>
+      <c r="AB4" s="4" t="n"/>
+      <c r="AC4" s="4" t="n"/>
+      <c r="AD4" s="4" t="n"/>
     </row>
     <row r="5">
       <c r="A5" s="3" t="n"/>
-      <c r="B5" s="3" t="inlineStr">
-        <is>
-          <t>Metrics</t>
-        </is>
-      </c>
+      <c r="B5" s="3" t="inlineStr"/>
       <c r="C5" s="4" t="inlineStr">
         <is>
           <t>beta</t>
@@ -1919,94 +1929,129 @@
           <t>CI_upper</t>
         </is>
       </c>
-      <c r="F5" s="3" t="inlineStr">
+      <c r="F5" s="4" t="inlineStr">
+        <is>
+          <t>CI Relative Width Ratio</t>
+        </is>
+      </c>
+      <c r="G5" s="3" t="inlineStr">
         <is>
           <t>beta</t>
         </is>
       </c>
-      <c r="G5" s="3" t="inlineStr">
+      <c r="H5" s="3" t="inlineStr">
         <is>
           <t>CI_lower</t>
         </is>
       </c>
-      <c r="H5" s="3" t="inlineStr">
+      <c r="I5" s="3" t="inlineStr">
         <is>
           <t>CI_upper</t>
         </is>
       </c>
-      <c r="I5" s="4" t="inlineStr">
+      <c r="J5" s="3" t="inlineStr">
+        <is>
+          <t>CI Relative Width Ratio</t>
+        </is>
+      </c>
+      <c r="K5" s="4" t="inlineStr">
         <is>
           <t>beta</t>
         </is>
       </c>
-      <c r="J5" s="4" t="inlineStr">
+      <c r="L5" s="4" t="inlineStr">
         <is>
           <t>CI_lower</t>
         </is>
       </c>
-      <c r="K5" s="4" t="inlineStr">
+      <c r="M5" s="4" t="inlineStr">
         <is>
           <t>CI_upper</t>
         </is>
       </c>
-      <c r="L5" s="3" t="inlineStr">
+      <c r="N5" s="4" t="inlineStr">
+        <is>
+          <t>CI Relative Width Ratio</t>
+        </is>
+      </c>
+      <c r="O5" s="3" t="inlineStr">
         <is>
           <t>beta</t>
         </is>
       </c>
-      <c r="M5" s="3" t="inlineStr">
+      <c r="P5" s="3" t="inlineStr">
         <is>
           <t>CI_lower</t>
         </is>
       </c>
-      <c r="N5" s="3" t="inlineStr">
+      <c r="Q5" s="3" t="inlineStr">
         <is>
           <t>CI_upper</t>
         </is>
       </c>
-      <c r="O5" s="4" t="inlineStr">
+      <c r="R5" s="3" t="inlineStr">
+        <is>
+          <t>CI Relative Width Ratio</t>
+        </is>
+      </c>
+      <c r="S5" s="4" t="inlineStr">
         <is>
           <t>beta</t>
         </is>
       </c>
-      <c r="P5" s="4" t="inlineStr">
+      <c r="T5" s="4" t="inlineStr">
         <is>
           <t>CI_lower</t>
         </is>
       </c>
-      <c r="Q5" s="4" t="inlineStr">
+      <c r="U5" s="4" t="inlineStr">
         <is>
           <t>CI_upper</t>
         </is>
       </c>
-      <c r="R5" s="3" t="inlineStr">
+      <c r="V5" s="4" t="inlineStr">
+        <is>
+          <t>CI Relative Width Ratio</t>
+        </is>
+      </c>
+      <c r="W5" s="3" t="inlineStr">
         <is>
           <t>beta</t>
         </is>
       </c>
-      <c r="S5" s="3" t="inlineStr">
+      <c r="X5" s="3" t="inlineStr">
         <is>
           <t>CI_lower</t>
         </is>
       </c>
-      <c r="T5" s="3" t="inlineStr">
+      <c r="Y5" s="3" t="inlineStr">
         <is>
           <t>CI_upper</t>
         </is>
       </c>
-      <c r="U5" s="4" t="inlineStr">
+      <c r="Z5" s="3" t="inlineStr">
+        <is>
+          <t>CI Relative Width Ratio</t>
+        </is>
+      </c>
+      <c r="AA5" s="4" t="inlineStr">
         <is>
           <t>beta</t>
         </is>
       </c>
-      <c r="V5" s="4" t="inlineStr">
+      <c r="AB5" s="4" t="inlineStr">
         <is>
           <t>CI_lower</t>
         </is>
       </c>
-      <c r="W5" s="4" t="inlineStr">
+      <c r="AC5" s="4" t="inlineStr">
         <is>
           <t>CI_upper</t>
+        </is>
+      </c>
+      <c r="AD5" s="4" t="inlineStr">
+        <is>
+          <t>CI Relative Width Ratio</t>
         </is>
       </c>
     </row>
@@ -2024,24 +2069,31 @@
       <c r="C6" s="4" t="n"/>
       <c r="D6" s="4" t="n"/>
       <c r="E6" s="4" t="n"/>
-      <c r="F6" s="3" t="n"/>
+      <c r="F6" s="4" t="n"/>
       <c r="G6" s="3" t="n"/>
       <c r="H6" s="3" t="n"/>
-      <c r="I6" s="4" t="n"/>
-      <c r="J6" s="4" t="n"/>
+      <c r="I6" s="3" t="n"/>
+      <c r="J6" s="3" t="n"/>
       <c r="K6" s="4" t="n"/>
-      <c r="L6" s="3" t="n"/>
-      <c r="M6" s="3" t="n"/>
-      <c r="N6" s="3" t="n"/>
-      <c r="O6" s="4" t="n"/>
-      <c r="P6" s="4" t="n"/>
-      <c r="Q6" s="4" t="n"/>
+      <c r="L6" s="4" t="n"/>
+      <c r="M6" s="4" t="n"/>
+      <c r="N6" s="4" t="n"/>
+      <c r="O6" s="3" t="n"/>
+      <c r="P6" s="3" t="n"/>
+      <c r="Q6" s="3" t="n"/>
       <c r="R6" s="3" t="n"/>
-      <c r="S6" s="3" t="n"/>
-      <c r="T6" s="3" t="n"/>
+      <c r="S6" s="4" t="n"/>
+      <c r="T6" s="4" t="n"/>
       <c r="U6" s="4" t="n"/>
       <c r="V6" s="4" t="n"/>
-      <c r="W6" s="4" t="n"/>
+      <c r="W6" s="3" t="n"/>
+      <c r="X6" s="3" t="n"/>
+      <c r="Y6" s="3" t="n"/>
+      <c r="Z6" s="3" t="n"/>
+      <c r="AA6" s="4" t="n"/>
+      <c r="AB6" s="4" t="n"/>
+      <c r="AC6" s="4" t="n"/>
+      <c r="AD6" s="4" t="n"/>
     </row>
     <row r="7">
       <c r="A7" s="4" t="inlineStr">
@@ -2064,58 +2116,79 @@
         <v>0.4452411736373632</v>
       </c>
       <c r="F7" s="5" t="n">
+        <v>3.624249494910925</v>
+      </c>
+      <c r="G7" s="5" t="n">
         <v>0.2618790981863163</v>
       </c>
-      <c r="G7" s="5" t="n">
+      <c r="H7" s="5" t="n">
         <v>-1.241497356439079</v>
       </c>
-      <c r="H7" s="5" t="n">
+      <c r="I7" s="5" t="n">
         <v>1.765255552811711</v>
       </c>
-      <c r="I7" s="5" t="n">
+      <c r="J7" s="5" t="n">
+        <v>11.48145434314734</v>
+      </c>
+      <c r="K7" s="5" t="n">
         <v>-1.968836043767184</v>
       </c>
-      <c r="J7" s="5" t="n">
+      <c r="L7" s="5" t="n">
         <v>-3.671718131445655</v>
       </c>
-      <c r="K7" s="5" t="n">
+      <c r="M7" s="5" t="n">
         <v>-0.2659539560887143</v>
       </c>
-      <c r="L7" s="5" t="n">
+      <c r="N7" s="5" t="n">
+        <v>1.729836359984718</v>
+      </c>
+      <c r="O7" s="5" t="n">
         <v>-1.08749923244575</v>
       </c>
-      <c r="M7" s="5" t="n">
+      <c r="P7" s="5" t="n">
         <v>-6.053568293348436</v>
       </c>
-      <c r="N7" s="5" t="n">
+      <c r="Q7" s="5" t="n">
         <v>3.878569828456935</v>
       </c>
-      <c r="O7" s="5" t="n">
+      <c r="R7" s="5" t="n">
+        <v>9.133007017824109</v>
+      </c>
+      <c r="S7" s="5" t="n">
         <v>-0.660968084728121</v>
       </c>
-      <c r="P7" s="5" t="n">
+      <c r="T7" s="5" t="n">
         <v>-2.597605518485457</v>
       </c>
-      <c r="Q7" s="5" t="n">
+      <c r="U7" s="5" t="n">
         <v>1.275669349029215</v>
       </c>
-      <c r="R7" s="5" t="n">
+      <c r="V7" s="5" t="n">
+        <v>5.860002860967007</v>
+      </c>
+      <c r="W7" s="5" t="n">
         <v>0.6992802674585527</v>
       </c>
-      <c r="S7" s="5" t="n">
+      <c r="X7" s="5" t="n">
         <v>-0.3296216144376013</v>
       </c>
-      <c r="T7" s="5" t="n">
+      <c r="Y7" s="5" t="n">
         <v>1.728182149354707</v>
       </c>
-      <c r="U7" s="5" t="n">
+      <c r="Z7" s="5" t="n">
+        <v>2.942745361986461</v>
+      </c>
+      <c r="AA7" s="5" t="n">
         <v>1.632130213666181</v>
       </c>
-      <c r="V7" s="5" t="n">
+      <c r="AB7" s="5" t="n">
         <v>-1.415682567705457</v>
       </c>
-      <c r="W7" s="5" t="n">
+      <c r="AC7" s="5" t="n">
         <v>4.67994299503782</v>
+      </c>
+      <c r="AD7" s="5" t="n">
+        <v>3.734766694289021</v>
       </c>
     </row>
     <row r="8">
@@ -2135,58 +2208,79 @@
         <v>0.0007795597253344524</v>
       </c>
       <c r="F8" s="5" t="n">
+        <v>3.71252241431292</v>
+      </c>
+      <c r="G8" s="5" t="n">
         <v>0.0002424318847966879</v>
       </c>
-      <c r="G8" s="5" t="n">
+      <c r="H8" s="5" t="n">
         <v>-0.00028465629453139</v>
       </c>
-      <c r="H8" s="5" t="n">
+      <c r="I8" s="5" t="n">
         <v>0.0007695200641247657</v>
       </c>
-      <c r="I8" s="5" t="n">
+      <c r="J8" s="5" t="n">
+        <v>4.348340398954643</v>
+      </c>
+      <c r="K8" s="5" t="n">
         <v>-0.0002745589580463794</v>
       </c>
-      <c r="J8" s="5" t="n">
+      <c r="L8" s="5" t="n">
         <v>-0.001166546185215082</v>
       </c>
-      <c r="K8" s="5" t="n">
+      <c r="M8" s="5" t="n">
         <v>0.0006174282691223228</v>
       </c>
-      <c r="L8" s="5" t="n">
+      <c r="N8" s="5" t="n">
+        <v>6.497600613839923</v>
+      </c>
+      <c r="O8" s="5" t="n">
         <v>-1.293322461919992e-06</v>
       </c>
-      <c r="M8" s="5" t="n">
+      <c r="P8" s="5" t="n">
         <v>-0.002713825801965323</v>
       </c>
-      <c r="N8" s="5" t="n">
+      <c r="Q8" s="5" t="n">
         <v>0.002711239157041483</v>
       </c>
-      <c r="O8" s="5" t="n">
+      <c r="R8" s="5" t="n">
+        <v>4194.673114200049</v>
+      </c>
+      <c r="S8" s="5" t="n">
         <v>0.0008794828932350875</v>
       </c>
-      <c r="P8" s="5" t="n">
+      <c r="T8" s="5" t="n">
         <v>-0.0003107812168985434</v>
       </c>
-      <c r="Q8" s="5" t="n">
+      <c r="U8" s="5" t="n">
         <v>0.002069747003368718</v>
       </c>
-      <c r="R8" s="5" t="n">
+      <c r="V8" s="5" t="n">
+        <v>2.70673624078205</v>
+      </c>
+      <c r="W8" s="5" t="n">
         <v>-0.0004406723349784292</v>
       </c>
-      <c r="S8" s="5" t="n">
+      <c r="X8" s="5" t="n">
         <v>-0.001223392685203437</v>
       </c>
-      <c r="T8" s="5" t="n">
+      <c r="Y8" s="5" t="n">
         <v>0.0003420480152465782</v>
       </c>
-      <c r="U8" s="5" t="n">
+      <c r="Z8" s="5" t="n">
+        <v>3.552391598457485</v>
+      </c>
+      <c r="AA8" s="5" t="n">
         <v>-0.0003112903627832451</v>
       </c>
-      <c r="V8" s="5" t="n">
+      <c r="AB8" s="5" t="n">
         <v>-0.00272779694097448</v>
       </c>
-      <c r="W8" s="5" t="n">
+      <c r="AC8" s="5" t="n">
         <v>0.00210521621540799</v>
+      </c>
+      <c r="AD8" s="5" t="n">
+        <v>15.52573974076978</v>
       </c>
     </row>
     <row r="9">
@@ -2209,59 +2303,80 @@
       <c r="E9" s="5" t="n">
         <v>0.01505899497979697</v>
       </c>
-      <c r="F9" s="6" t="n">
+      <c r="F9" s="5" t="n">
+        <v>4.500684972021411</v>
+      </c>
+      <c r="G9" s="6" t="n">
         <v>-0.003217276961140139</v>
       </c>
-      <c r="G9" s="6" t="n">
+      <c r="H9" s="6" t="n">
         <v>-0.03032001839346419</v>
       </c>
-      <c r="H9" s="6" t="n">
+      <c r="I9" s="6" t="n">
         <v>0.02388546447118392</v>
       </c>
-      <c r="I9" s="5" t="n">
+      <c r="J9" s="6" t="n">
+        <v>16.84824885123933</v>
+      </c>
+      <c r="K9" s="5" t="n">
         <v>-0.01354486073883431</v>
       </c>
-      <c r="J9" s="5" t="n">
+      <c r="L9" s="5" t="n">
         <v>-0.05586486084421864</v>
       </c>
-      <c r="K9" s="5" t="n">
+      <c r="M9" s="5" t="n">
         <v>0.02877513936655002</v>
       </c>
-      <c r="L9" s="6" t="n">
+      <c r="N9" s="5" t="n">
+        <v>6.248864557765317</v>
+      </c>
+      <c r="O9" s="6" t="n">
         <v>-0.05676428376993873</v>
       </c>
-      <c r="M9" s="6" t="n">
+      <c r="P9" s="6" t="n">
         <v>-0.146027198396996</v>
       </c>
-      <c r="N9" s="6" t="n">
+      <c r="Q9" s="6" t="n">
         <v>0.03249863085711849</v>
       </c>
-      <c r="O9" s="5" t="n">
+      <c r="R9" s="6" t="n">
+        <v>3.145037995681684</v>
+      </c>
+      <c r="S9" s="5" t="n">
         <v>-0.04954613454682324</v>
       </c>
-      <c r="P9" s="5" t="n">
+      <c r="T9" s="5" t="n">
         <v>-0.1069826481655368</v>
       </c>
-      <c r="Q9" s="5" t="n">
+      <c r="U9" s="5" t="n">
         <v>0.007890379071890309</v>
       </c>
-      <c r="R9" s="6" t="n">
+      <c r="V9" s="5" t="n">
+        <v>2.31850634339329</v>
+      </c>
+      <c r="W9" s="6" t="n">
         <v>0.02272648726281115</v>
       </c>
-      <c r="S9" s="6" t="n">
+      <c r="X9" s="6" t="n">
         <v>-0.006496658296303331</v>
       </c>
-      <c r="T9" s="6" t="n">
+      <c r="Y9" s="6" t="n">
         <v>0.05194963282192563</v>
       </c>
-      <c r="U9" s="5" t="n">
+      <c r="Z9" s="6" t="n">
+        <v>2.57172568916396</v>
+      </c>
+      <c r="AA9" s="5" t="n">
         <v>0.001779703779848962</v>
       </c>
-      <c r="V9" s="5" t="n">
+      <c r="AB9" s="5" t="n">
         <v>-0.04672758840926379</v>
       </c>
-      <c r="W9" s="5" t="n">
+      <c r="AC9" s="5" t="n">
         <v>0.05028699596896172</v>
+      </c>
+      <c r="AD9" s="5" t="n">
+        <v>54.51164709357355</v>
       </c>
     </row>
     <row r="10">
@@ -2285,58 +2400,79 @@
         <v>0.0004570939405830946</v>
       </c>
       <c r="F10" s="5" t="n">
+        <v>3.884155804448329</v>
+      </c>
+      <c r="G10" s="5" t="n">
         <v>-0.000826195660979923</v>
       </c>
-      <c r="G10" s="5" t="n">
+      <c r="H10" s="5" t="n">
         <v>-0.002517082529766342</v>
       </c>
-      <c r="H10" s="5" t="n">
+      <c r="I10" s="5" t="n">
         <v>0.0008646912078064965</v>
       </c>
-      <c r="I10" s="5" t="n">
+      <c r="J10" s="5" t="n">
+        <v>4.093187482444328</v>
+      </c>
+      <c r="K10" s="5" t="n">
         <v>-0.001001619124555685</v>
       </c>
-      <c r="J10" s="5" t="n">
+      <c r="L10" s="5" t="n">
         <v>-0.002973321477981247</v>
       </c>
-      <c r="K10" s="5" t="n">
+      <c r="M10" s="5" t="n">
         <v>0.0009700832288698775</v>
       </c>
-      <c r="L10" s="5" t="n">
+      <c r="N10" s="5" t="n">
+        <v>3.937030164635092</v>
+      </c>
+      <c r="O10" s="5" t="n">
         <v>0.0006516030606860851</v>
       </c>
-      <c r="M10" s="5" t="n">
+      <c r="P10" s="5" t="n">
         <v>-0.002247059131435814</v>
       </c>
-      <c r="N10" s="5" t="n">
+      <c r="Q10" s="5" t="n">
         <v>0.003550265252807984</v>
       </c>
-      <c r="O10" s="5" t="n">
+      <c r="R10" s="5" t="n">
+        <v>8.897018344480589</v>
+      </c>
+      <c r="S10" s="5" t="n">
         <v>-4.948763045824571e-05</v>
       </c>
-      <c r="P10" s="5" t="n">
+      <c r="T10" s="5" t="n">
         <v>-0.002475607803393917</v>
       </c>
-      <c r="Q10" s="5" t="n">
+      <c r="U10" s="5" t="n">
         <v>0.002376632542477425</v>
       </c>
-      <c r="R10" s="5" t="n">
+      <c r="V10" s="5" t="n">
+        <v>98.04955907042935</v>
+      </c>
+      <c r="W10" s="5" t="n">
         <v>-0.0002660068688006391</v>
       </c>
-      <c r="S10" s="5" t="n">
+      <c r="X10" s="5" t="n">
         <v>-0.001611860824041869</v>
       </c>
-      <c r="T10" s="5" t="n">
+      <c r="Y10" s="5" t="n">
         <v>0.001079847086440591</v>
       </c>
-      <c r="U10" s="5" t="n">
+      <c r="Z10" s="5" t="n">
+        <v>10.11894137402813</v>
+      </c>
+      <c r="AA10" s="5" t="n">
         <v>-0.002713913057161963</v>
       </c>
-      <c r="V10" s="5" t="n">
+      <c r="AB10" s="5" t="n">
         <v>-0.006561771854417833</v>
       </c>
-      <c r="W10" s="5" t="n">
+      <c r="AC10" s="5" t="n">
         <v>0.001133945740093906</v>
+      </c>
+      <c r="AD10" s="5" t="n">
+        <v>2.835653697233554</v>
       </c>
     </row>
     <row r="11">
@@ -2359,59 +2495,80 @@
       <c r="E11" s="5" t="n">
         <v>0.02693719132326763</v>
       </c>
-      <c r="F11" s="6" t="n">
+      <c r="F11" s="5" t="n">
+        <v>20.95140988269725</v>
+      </c>
+      <c r="G11" s="6" t="n">
         <v>0.01896011281041776</v>
       </c>
-      <c r="G11" s="6" t="n">
+      <c r="H11" s="6" t="n">
         <v>-0.007808068322245926</v>
       </c>
-      <c r="H11" s="6" t="n">
+      <c r="I11" s="6" t="n">
         <v>0.04572829394308144</v>
       </c>
-      <c r="I11" s="5" t="n">
+      <c r="J11" s="6" t="n">
+        <v>2.823630998435382</v>
+      </c>
+      <c r="K11" s="5" t="n">
         <v>0.01110720076736025</v>
       </c>
-      <c r="J11" s="5" t="n">
+      <c r="L11" s="5" t="n">
         <v>-0.01827997127370456</v>
       </c>
-      <c r="K11" s="5" t="n">
+      <c r="M11" s="5" t="n">
         <v>0.04049437280842505</v>
       </c>
-      <c r="L11" s="6" t="n">
+      <c r="N11" s="5" t="n">
+        <v>5.291553228680678</v>
+      </c>
+      <c r="O11" s="6" t="n">
         <v>-0.05688451707978919</v>
       </c>
-      <c r="M11" s="6" t="n">
+      <c r="P11" s="6" t="n">
         <v>-0.1198278250631943</v>
       </c>
-      <c r="N11" s="6" t="n">
+      <c r="Q11" s="6" t="n">
         <v>0.006058790903615906</v>
       </c>
-      <c r="O11" s="5" t="n">
+      <c r="R11" s="6" t="n">
+        <v>2.213020737966977</v>
+      </c>
+      <c r="S11" s="5" t="n">
         <v>0.001783838005130882</v>
       </c>
-      <c r="P11" s="5" t="n">
+      <c r="T11" s="5" t="n">
         <v>-0.03840240777512716</v>
       </c>
-      <c r="Q11" s="5" t="n">
+      <c r="U11" s="5" t="n">
         <v>0.04197008378538893</v>
       </c>
-      <c r="R11" s="6" t="n">
+      <c r="V11" s="5" t="n">
+        <v>45.05593631783795</v>
+      </c>
+      <c r="W11" s="6" t="n">
         <v>-0.03251854003148871</v>
       </c>
-      <c r="S11" s="6" t="n">
+      <c r="X11" s="6" t="n">
         <v>-0.06073261868674925</v>
       </c>
-      <c r="T11" s="6" t="n">
+      <c r="Y11" s="6" t="n">
         <v>-0.004304461376228162</v>
       </c>
-      <c r="U11" s="5" t="n">
+      <c r="Z11" s="6" t="n">
+        <v>1.735261092775997</v>
+      </c>
+      <c r="AA11" s="5" t="n">
         <v>-0.01889481480612774</v>
       </c>
-      <c r="V11" s="5" t="n">
+      <c r="AB11" s="5" t="n">
         <v>-0.07735891032834516</v>
       </c>
-      <c r="W11" s="5" t="n">
+      <c r="AC11" s="5" t="n">
         <v>0.03956928071608967</v>
+      </c>
+      <c r="AD11" s="5" t="n">
+        <v>6.188374548477398</v>
       </c>
     </row>
     <row r="12">
@@ -2430,59 +2587,80 @@
       <c r="E12" s="5" t="n">
         <v>-0.0048536665101706</v>
       </c>
-      <c r="F12" s="6" t="n">
+      <c r="F12" s="5" t="n">
+        <v>1.474084632164657</v>
+      </c>
+      <c r="G12" s="6" t="n">
         <v>-0.01648583523094233</v>
       </c>
-      <c r="G12" s="6" t="n">
+      <c r="H12" s="6" t="n">
         <v>-0.0314190116494683</v>
       </c>
-      <c r="H12" s="6" t="n">
+      <c r="I12" s="6" t="n">
         <v>-0.001552658812416365</v>
       </c>
-      <c r="I12" s="5" t="n">
+      <c r="J12" s="6" t="n">
+        <v>1.811637227878856</v>
+      </c>
+      <c r="K12" s="5" t="n">
         <v>0.01691014377155839</v>
       </c>
-      <c r="J12" s="5" t="n">
+      <c r="L12" s="5" t="n">
         <v>-0.0108958720644927</v>
       </c>
-      <c r="K12" s="5" t="n">
+      <c r="M12" s="5" t="n">
         <v>0.04471615960760948</v>
       </c>
-      <c r="L12" s="6" t="n">
+      <c r="N12" s="5" t="n">
+        <v>3.288678820438979</v>
+      </c>
+      <c r="O12" s="6" t="n">
         <v>-0.04879046560426468</v>
       </c>
-      <c r="M12" s="6" t="n">
+      <c r="P12" s="6" t="n">
         <v>-0.09136952139527177</v>
       </c>
-      <c r="N12" s="6" t="n">
+      <c r="Q12" s="6" t="n">
         <v>-0.006211409813257594</v>
       </c>
-      <c r="O12" s="5" t="n">
+      <c r="R12" s="6" t="n">
+        <v>1.745384278000632</v>
+      </c>
+      <c r="S12" s="5" t="n">
         <v>-0.002082114571569562</v>
       </c>
-      <c r="P12" s="5" t="n">
+      <c r="T12" s="5" t="n">
         <v>-0.03856735295211186</v>
       </c>
-      <c r="Q12" s="5" t="n">
+      <c r="U12" s="5" t="n">
         <v>0.03440312380897273</v>
       </c>
-      <c r="R12" s="6" t="n">
+      <c r="V12" s="5" t="n">
+        <v>35.04633114693453</v>
+      </c>
+      <c r="W12" s="6" t="n">
         <v>-0.01246091850018913</v>
       </c>
-      <c r="S12" s="6" t="n">
+      <c r="X12" s="6" t="n">
         <v>-0.02924813469244573</v>
       </c>
-      <c r="T12" s="6" t="n">
+      <c r="Y12" s="6" t="n">
         <v>0.004326297692067462</v>
       </c>
-      <c r="U12" s="5" t="n">
+      <c r="Z12" s="6" t="n">
+        <v>2.694378619361293</v>
+      </c>
+      <c r="AA12" s="5" t="n">
         <v>-0.06684304493937422</v>
       </c>
-      <c r="V12" s="5" t="n">
+      <c r="AB12" s="5" t="n">
         <v>-0.1035095475778177</v>
       </c>
-      <c r="W12" s="5" t="n">
+      <c r="AC12" s="5" t="n">
         <v>-0.0301765423009307</v>
+      </c>
+      <c r="AD12" s="5" t="n">
+        <v>1.097092529872018</v>
       </c>
     </row>
     <row r="13">
@@ -2506,58 +2684,79 @@
         <v>-0.1365616983555663</v>
       </c>
       <c r="F13" s="5" t="n">
+        <v>1.21509316857662</v>
+      </c>
+      <c r="G13" s="5" t="n">
         <v>-0.554850971333216</v>
       </c>
-      <c r="G13" s="5" t="n">
+      <c r="H13" s="5" t="n">
         <v>-0.8809675042797518</v>
       </c>
-      <c r="H13" s="5" t="n">
+      <c r="I13" s="5" t="n">
         <v>-0.2287344383866802</v>
       </c>
-      <c r="I13" s="5" t="n">
+      <c r="J13" s="5" t="n">
+        <v>1.175510361504572</v>
+      </c>
+      <c r="K13" s="5" t="n">
         <v>-0.04378003435391339</v>
       </c>
-      <c r="J13" s="5" t="n">
+      <c r="L13" s="5" t="n">
         <v>-0.4557753430651801</v>
       </c>
-      <c r="K13" s="5" t="n">
+      <c r="M13" s="5" t="n">
         <v>0.3682152743573534</v>
       </c>
-      <c r="L13" s="5" t="n">
+      <c r="N13" s="5" t="n">
+        <v>18.82115054459474</v>
+      </c>
+      <c r="O13" s="5" t="n">
         <v>-0.06869547448332119</v>
       </c>
-      <c r="M13" s="5" t="n">
+      <c r="P13" s="5" t="n">
         <v>-0.7660613520725512</v>
       </c>
-      <c r="N13" s="5" t="n">
+      <c r="Q13" s="5" t="n">
         <v>0.6286704031059089</v>
       </c>
-      <c r="O13" s="5" t="n">
+      <c r="R13" s="5" t="n">
+        <v>20.30310971237402</v>
+      </c>
+      <c r="S13" s="5" t="n">
         <v>-0.06961261982621557</v>
       </c>
-      <c r="P13" s="5" t="n">
+      <c r="T13" s="5" t="n">
         <v>-0.5769174265387652</v>
       </c>
-      <c r="Q13" s="5" t="n">
+      <c r="U13" s="5" t="n">
         <v>0.437692186886334</v>
       </c>
-      <c r="R13" s="5" t="n">
+      <c r="V13" s="5" t="n">
+        <v>14.57508158661492</v>
+      </c>
+      <c r="W13" s="5" t="n">
         <v>0.03657371716226639</v>
       </c>
-      <c r="S13" s="5" t="n">
+      <c r="X13" s="5" t="n">
         <v>-0.3564487731097409</v>
       </c>
-      <c r="T13" s="5" t="n">
+      <c r="Y13" s="5" t="n">
         <v>0.4295962074342737</v>
       </c>
-      <c r="U13" s="5" t="n">
+      <c r="Z13" s="5" t="n">
+        <v>21.4920724917452</v>
+      </c>
+      <c r="AA13" s="5" t="n">
         <v>0.4663416192881011</v>
       </c>
-      <c r="V13" s="5" t="n">
+      <c r="AB13" s="5" t="n">
         <v>-0.2860530578119991</v>
       </c>
-      <c r="W13" s="5" t="n">
+      <c r="AC13" s="5" t="n">
         <v>1.218736296388201</v>
+      </c>
+      <c r="AD13" s="5" t="n">
+        <v>3.226796176797072</v>
       </c>
     </row>
     <row r="14">
@@ -2580,59 +2779,80 @@
       <c r="E14" s="5" t="n">
         <v>0.0009210863419540222</v>
       </c>
-      <c r="F14" s="6" t="n">
+      <c r="F14" s="5" t="n">
+        <v>2.041156055929885</v>
+      </c>
+      <c r="G14" s="6" t="n">
         <v>-0.03101491007731285</v>
       </c>
-      <c r="G14" s="6" t="n">
+      <c r="H14" s="6" t="n">
         <v>-0.1047056127809043</v>
       </c>
-      <c r="H14" s="6" t="n">
+      <c r="I14" s="6" t="n">
         <v>0.04267579262627855</v>
       </c>
-      <c r="I14" s="5" t="n">
+      <c r="J14" s="6" t="n">
+        <v>4.751953335985684</v>
+      </c>
+      <c r="K14" s="5" t="n">
         <v>-0.03388319657228572</v>
       </c>
-      <c r="J14" s="5" t="n">
+      <c r="L14" s="5" t="n">
         <v>-0.1395923685113756</v>
       </c>
-      <c r="K14" s="5" t="n">
+      <c r="M14" s="5" t="n">
         <v>0.07182597536680418</v>
       </c>
-      <c r="L14" s="6" t="n">
+      <c r="N14" s="5" t="n">
+        <v>6.239622150972216</v>
+      </c>
+      <c r="O14" s="6" t="n">
         <v>0.0472199908514435</v>
       </c>
-      <c r="M14" s="6" t="n">
+      <c r="P14" s="6" t="n">
         <v>-0.1055560673899905</v>
       </c>
-      <c r="N14" s="6" t="n">
+      <c r="Q14" s="6" t="n">
         <v>0.1999960490928775</v>
       </c>
-      <c r="O14" s="5" t="n">
+      <c r="R14" s="6" t="n">
+        <v>6.470821170723021</v>
+      </c>
+      <c r="S14" s="5" t="n">
         <v>-0.03480524597027135</v>
       </c>
-      <c r="P14" s="5" t="n">
+      <c r="T14" s="5" t="n">
         <v>-0.1666050098385253</v>
       </c>
-      <c r="Q14" s="5" t="n">
+      <c r="U14" s="5" t="n">
         <v>0.09699451789798258</v>
       </c>
-      <c r="R14" s="6" t="n">
+      <c r="V14" s="5" t="n">
+        <v>7.573557387344986</v>
+      </c>
+      <c r="W14" s="6" t="n">
         <v>0.0281414002973919</v>
       </c>
-      <c r="S14" s="6" t="n">
+      <c r="X14" s="6" t="n">
         <v>-0.02594265594952315</v>
       </c>
-      <c r="T14" s="6" t="n">
+      <c r="Y14" s="6" t="n">
         <v>0.08222545654430695</v>
       </c>
-      <c r="U14" s="5" t="n">
+      <c r="Z14" s="6" t="n">
+        <v>3.843735967319826</v>
+      </c>
+      <c r="AA14" s="5" t="n">
         <v>0.08674972761160121</v>
       </c>
-      <c r="V14" s="5" t="n">
+      <c r="AB14" s="5" t="n">
         <v>-0.06970115338726085</v>
       </c>
-      <c r="W14" s="5" t="n">
+      <c r="AC14" s="5" t="n">
         <v>0.2432006086104633</v>
+      </c>
+      <c r="AD14" s="5" t="n">
+        <v>3.606948063268375</v>
       </c>
     </row>
     <row r="15">
@@ -2651,75 +2871,96 @@
       <c r="E15" s="5" t="n">
         <v>0.05548067379963971</v>
       </c>
-      <c r="F15" s="6" t="n">
+      <c r="F15" s="5" t="n">
+        <v>4.159371044652015</v>
+      </c>
+      <c r="G15" s="6" t="n">
         <v>0.02394157441402341</v>
       </c>
-      <c r="G15" s="6" t="n">
+      <c r="H15" s="6" t="n">
         <v>-0.03469264895659442</v>
       </c>
-      <c r="H15" s="6" t="n">
+      <c r="I15" s="6" t="n">
         <v>0.08257579778464123</v>
       </c>
-      <c r="I15" s="5" t="n">
+      <c r="J15" s="6" t="n">
+        <v>4.898109235144847</v>
+      </c>
+      <c r="K15" s="5" t="n">
         <v>0.1940446307095657</v>
       </c>
-      <c r="J15" s="5" t="n">
+      <c r="L15" s="5" t="n">
         <v>0.02720669959656918</v>
       </c>
-      <c r="K15" s="5" t="n">
+      <c r="M15" s="5" t="n">
         <v>0.3608825618225622</v>
       </c>
-      <c r="L15" s="6" t="n">
+      <c r="N15" s="5" t="n">
+        <v>1.719583072233619</v>
+      </c>
+      <c r="O15" s="6" t="n">
         <v>0.06746046882238525</v>
       </c>
-      <c r="M15" s="6" t="n">
+      <c r="P15" s="6" t="n">
         <v>-0.08277076473970842</v>
       </c>
-      <c r="N15" s="6" t="n">
+      <c r="Q15" s="6" t="n">
         <v>0.2176917023844789</v>
       </c>
-      <c r="O15" s="5" t="n">
+      <c r="R15" s="6" t="n">
+        <v>4.453904225232505</v>
+      </c>
+      <c r="S15" s="5" t="n">
         <v>0.132076941747987</v>
       </c>
-      <c r="P15" s="5" t="n">
+      <c r="T15" s="5" t="n">
         <v>0.04811570527043092</v>
       </c>
-      <c r="Q15" s="5" t="n">
+      <c r="U15" s="5" t="n">
         <v>0.2160381782255432</v>
       </c>
-      <c r="R15" s="6" t="n">
+      <c r="V15" s="5" t="n">
+        <v>1.271398858367884</v>
+      </c>
+      <c r="W15" s="6" t="n">
         <v>0.02793195311850622</v>
       </c>
-      <c r="S15" s="6" t="n">
+      <c r="X15" s="6" t="n">
         <v>-0.02097406715310803</v>
       </c>
-      <c r="T15" s="6" t="n">
+      <c r="Y15" s="6" t="n">
         <v>0.07683797339012048</v>
       </c>
-      <c r="U15" s="5" t="n">
+      <c r="Z15" s="6" t="n">
+        <v>3.501797390545649</v>
+      </c>
+      <c r="AA15" s="5" t="n">
         <v>-0.1083130738338397</v>
       </c>
-      <c r="V15" s="5" t="n">
+      <c r="AB15" s="5" t="n">
         <v>-0.2215082881820247</v>
       </c>
-      <c r="W15" s="5" t="n">
+      <c r="AC15" s="5" t="n">
         <v>0.004882140514345226</v>
+      </c>
+      <c r="AD15" s="5" t="n">
+        <v>2.090148683654474</v>
       </c>
     </row>
   </sheetData>
   <mergeCells count="12">
-    <mergeCell ref="A1:W1"/>
+    <mergeCell ref="K4:N4"/>
+    <mergeCell ref="O4:R4"/>
+    <mergeCell ref="S4:V4"/>
+    <mergeCell ref="C4:F4"/>
     <mergeCell ref="A14:A15"/>
-    <mergeCell ref="O4:Q4"/>
-    <mergeCell ref="R4:T4"/>
-    <mergeCell ref="C4:E4"/>
-    <mergeCell ref="U4:W4"/>
-    <mergeCell ref="F4:H4"/>
+    <mergeCell ref="G4:J4"/>
+    <mergeCell ref="W4:Z4"/>
+    <mergeCell ref="AA4:AD4"/>
     <mergeCell ref="A7:A8"/>
-    <mergeCell ref="I4:K4"/>
-    <mergeCell ref="L4:N4"/>
-    <mergeCell ref="A2:W2"/>
+    <mergeCell ref="A2:AD2"/>
     <mergeCell ref="A11:A12"/>
+    <mergeCell ref="A1:AD1"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>